<commit_message>
docs: atualizacao com headwinds operacionais
</commit_message>
<xml_diff>
--- a/outputs/gmat3_valuation_research_workbook.xlsx
+++ b/outputs/gmat3_valuation_research_workbook.xlsx
@@ -24,13 +24,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="R$0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0x"/>
     <numFmt numFmtId="167" formatCode="R$#,##0"/>
+    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="169" formatCode="R$#,##0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,6 +75,11 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -102,7 +109,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -124,11 +131,55 @@
         <color rgb="00A6A6A6"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00A6A6A6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00A6A6A6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00A6A6A6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00A6A6A6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00A6A6A6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00A6A6A6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00A6A6A6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00A6A6A6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -188,6 +239,26 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -734,9 +805,9 @@
       <c r="H2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Tese: GMAT3 parece levemente descontada contra um peer set LatAm saudavel, mas nao e uma tese agressiva. GPA entra como stress/turnaround, nao como benchmark central.</t>
+      <c r="A3" s="23" t="inlineStr">
+        <is>
+          <t>Tese: GMAT3 parece moderadamente descontada frente a peers LatAm saudáveis, mas o 1T26 reduz a convicção por SSS negativo, deflação alimentar e trade-off entre margem e volume.</t>
         </is>
       </c>
     </row>
@@ -2003,7 +2074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2017,6 +2088,7 @@
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="45" customWidth="1" min="10" max="10"/>
     <col width="48" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2095,6 +2167,11 @@
           <t>Metodologia</t>
         </is>
       </c>
+      <c r="L3" s="24" t="inlineStr">
+        <is>
+          <t>Leitura qualitativa</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -2138,6 +2215,11 @@
           <t>25th percentile of full traded peer set, including GPA</t>
         </is>
       </c>
+      <c r="L4" s="25" t="inlineStr">
+        <is>
+          <t>Stress case: downside risk if weak SSS and margin pressure persist.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -2181,6 +2263,11 @@
           <t>Median of Brazilian listed peers, including distressed GPA</t>
         </is>
       </c>
+      <c r="L5" s="25" t="inlineStr">
+        <is>
+          <t>Stress case: downside risk if weak SSS and margin pressure persist.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -2224,6 +2311,11 @@
           <t>Assai-only case as closest domestic listed comparable</t>
         </is>
       </c>
+      <c r="L6" s="25" t="inlineStr">
+        <is>
+          <t>Scenario output should be interpreted with 1T26 operating caution.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -2267,6 +2359,11 @@
           <t>Median of traded peers excluding distressed GPA and delisted Carrefour Brasil</t>
         </is>
       </c>
+      <c r="L7" s="25" t="inlineStr">
+        <is>
+          <t>Base case: moderate upside, but operational caution required.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -2310,6 +2407,11 @@
           <t>Median of all traded peers, including GPA</t>
         </is>
       </c>
+      <c r="L8" s="25" t="inlineStr">
+        <is>
+          <t>Scenario output should be interpreted with 1T26 operating caution.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -2351,6 +2453,11 @@
       <c r="K9" s="7" t="inlineStr">
         <is>
           <t>Higher of GMAT3 current EV/EBITDA and ex-distressed peer 75th percentile</t>
+        </is>
+      </c>
+      <c r="L9" s="25" t="inlineStr">
+        <is>
+          <t>Bull case: upside increases if SSS normalizes and margin protection continues.</t>
         </is>
       </c>
     </row>
@@ -2387,13 +2494,13 @@
           <t>Lucro Liquido Setorial</t>
         </is>
       </c>
-      <c r="B1" s="18" t="n"/>
-      <c r="C1" s="18" t="n"/>
-      <c r="D1" s="18" t="n"/>
-      <c r="E1" s="18" t="n"/>
-      <c r="F1" s="18" t="n"/>
-      <c r="G1" s="18" t="n"/>
-      <c r="H1" s="18" t="n"/>
+      <c r="B1" s="26" t="n"/>
+      <c r="C1" s="26" t="n"/>
+      <c r="D1" s="26" t="n"/>
+      <c r="E1" s="26" t="n"/>
+      <c r="F1" s="26" t="n"/>
+      <c r="G1" s="26" t="n"/>
+      <c r="H1" s="27" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="18" t="n"/>
@@ -2411,13 +2518,13 @@
           <t>Lucro liquido setorial calculado separadamente para Brasil em BRL milhões. Nao somamos LatAm porque Walmex, Chedraui, Soriana e Cencosud reportam em outras moedas.</t>
         </is>
       </c>
-      <c r="B3" s="18" t="n"/>
-      <c r="C3" s="18" t="n"/>
-      <c r="D3" s="18" t="n"/>
-      <c r="E3" s="18" t="n"/>
-      <c r="F3" s="18" t="n"/>
-      <c r="G3" s="18" t="n"/>
-      <c r="H3" s="18" t="n"/>
+      <c r="B3" s="26" t="n"/>
+      <c r="C3" s="26" t="n"/>
+      <c r="D3" s="26" t="n"/>
+      <c r="E3" s="26" t="n"/>
+      <c r="F3" s="26" t="n"/>
+      <c r="G3" s="26" t="n"/>
+      <c r="H3" s="27" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="18" t="n"/>
@@ -2841,15 +2948,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="25" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
@@ -2858,214 +2965,396 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Tese Operacional</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Overlay Operacional 1T26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Pilar</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Argumento</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Por que importa</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Evidencia a buscar</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Risco</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Como falar</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Crescimento regional</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>GMAT3 tem posicao forte em mercados regionais, especialmente Norte/Nordeste.</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Conhecimento local e densidade operacional podem sustentar crescimento.</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>Aberturas, vendas mesmas lojas e market share regional.</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>Expansao fora do core pode reduzir retorno.</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>Forca regional sustenta premio relativo.</t>
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>O valuation aponta upside moderado, mas os dados operacionais do 1T26 reduzem a convicção. O ponto central é que a empresa protegeu margem bruta, mas sofreu com SSS negativo, deflação alimentar e desalavancagem operacional.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Maturacao de lojas</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Lojas recentes podem ganhar venda e margem ao longo do tempo.</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Crescimento nao depende apenas de novas lojas.</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Curva de maturacao e produtividade por loja.</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>Maturacao abaixo do esperado reduz EBITDA.</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Parte do upside vem de lojas amadurecendo.</t>
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>Métrica</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
+        <is>
+          <t>Leitura</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>Impacto na tese</t>
+        </is>
+      </c>
+      <c r="F5" s="24" t="inlineStr">
+        <is>
+          <t>Mensagem para apresentação</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Logistica e distribuicao</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Varejo alimentar depende de abastecimento eficiente.</t>
-        </is>
+          <t>Net revenue growth YoY</t>
+        </is>
+      </c>
+      <c r="B6" s="29" t="n">
+        <v>12.9</v>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Boa distribuicao reduz ruptura e custo.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>CDs, capilaridade, giro de estoque.</t>
+          <t>Revenue still grew, helped by consolidation and channel growth.</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Custo logistico e execucao regional.</t>
+          <t>Positivo, mas não suficiente para compensar pressão de lucro.</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Logistica e vantagem competitiva operacional.</t>
+          <t>Upside existe, mas precisa ser lido com cautela operacional.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Margem EBITDA</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Mercado paga mais por crescimento com margem resiliente.</t>
-        </is>
+          <t>Net income growth YoY</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="n">
+        <v>-21.8</v>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Multiplo precisa ser sustentado por rentabilidade.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Margem GMAT3 vs Assai/LatAm.</t>
+          <t>Profitability deteriorated despite revenue growth.</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Promocao e competicao pressionam margem.</t>
+          <t>Negativo para convicção de curto prazo.</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Sem margem, nao ha re-rating.</t>
+          <t>Upside existe, mas precisa ser lido com cautela operacional.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Competicao no atacarejo</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Assai, Atacadao e regionais disputam preco e trafego.</t>
-        </is>
+          <t>Same-store sales growth</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="n">
+        <v>-7.3</v>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Setor e competitivo e sensivel a preco.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Preco, abertura de lojas concorrentes, margem bruta.</t>
+          <t>Negative SSS points to weaker mature-store momentum.</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Guerra de preco.</t>
+          <t>Principal alerta operacional.</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Principal risco da tese.</t>
+          <t>Upside existe, mas precisa ser lido com cautela operacional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Gross margin</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Margin protection worked at the gross profit level.</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Mostra preservação de margem.</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Upside existe, mas precisa ser lido com cautela operacional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>EBITDA margin pre-IFRS 16</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Pre-IFRS profitability remains pressured.</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Mostra pressão operacional antes do efeito IFRS 16.</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Upside existe, mas precisa ser lido com cautela operacional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>EBITDA margin post-IFRS 16</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Post-IFRS 16 EBITDA margin also declined YoY.</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Margem reportada ainda pressionada.</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Upside existe, mas precisa ser lido com cautela operacional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>EBITDA pre-IFRS 16</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="n">
+        <v>399.8</v>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>BRL mn</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Used as an operating quality reference versus annualized EBITDA.</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Base operacional mais conservadora.</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Upside existe, mas precisa ser lido com cautela operacional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>EBITDA post-IFRS 16</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="n">
+        <v>543</v>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>BRL mn</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Reported post-IFRS EBITDA reference.</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Referência reportada pós-arrendamento.</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Upside existe, mas precisa ser lido com cautela operacional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>Pilar operacional</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>Tese</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="inlineStr">
+        <is>
+          <t>Risco</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Crescimento regional</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Força regional ainda sustenta a tese estrutural.</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Expansão fora do core pode reduzir retorno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Maturação de lojas</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Normalização de SSS é chave para o re-rating.</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>SSS negativo prolongado limita upside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Logística e distribuição</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Eficiência logística pode proteger margem.</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Custo logístico e ruptura podem pressionar rentabilidade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Margem EBITDA</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Preservação de margem é positiva, mas não pode depender de queda de volume.</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Trade-off margem vs volume reduz qualidade do crescimento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Competição no atacarejo</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Setor segue estruturalmente relevante.</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Assaí, Atacadão e players regionais pressionam preços.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A3:F3"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3078,7 +3367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3087,8 +3376,8 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="58" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="45" customWidth="1" min="10" max="10"/>
     <col width="48" customWidth="1" min="11" max="11"/>
@@ -3102,42 +3391,42 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="24" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="24" t="inlineStr">
         <is>
           <t>Empresa</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="24" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="24" t="inlineStr">
         <is>
           <t>Periodo/Data</t>
         </is>
       </c>
-      <c r="F3" s="14" t="inlineStr">
+      <c r="F3" s="24" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="24" t="inlineStr">
         <is>
           <t>Fonte</t>
         </is>
       </c>
-      <c r="H3" s="14" t="inlineStr">
+      <c r="H3" s="24" t="inlineStr">
         <is>
           <t>Uso</t>
         </is>
@@ -3285,7 +3574,9 @@
           <t>Expanded peer group</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n"/>
+      <c r="D7" s="7" t="n">
+        <v/>
+      </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
           <t>2026-05-31</t>
@@ -3407,7 +3698,9 @@
           <t>All peers</t>
         </is>
       </c>
-      <c r="D10" s="7" t="n"/>
+      <c r="D10" s="7" t="n">
+        <v/>
+      </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
           <t>2026-05-31</t>
@@ -3426,6 +3719,48 @@
       <c r="H10" s="7" t="inlineStr">
         <is>
           <t>Peer group classification</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>SRC008</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>1T26 operating evidence</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Grupo Mateus</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>GMAT3.SA</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>News / earnings analysis</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>https://www.moneytimes.com.br/grupo-mateus-gmat3-ve-lucro-cair-218-no-1t26-para-r-2129-milhoes/</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Operational overlay and risk interpretation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add LTM methodology outputs and equity research report for GMAT3
</commit_message>
<xml_diff>
--- a/outputs/gmat3_valuation_research_workbook.xlsx
+++ b/outputs/gmat3_valuation_research_workbook.xlsx
@@ -35,7 +35,7 @@
     <numFmt numFmtId="168" formatCode="0.0"/>
     <numFmt numFmtId="169" formatCode="R$#,##0.0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,6 +87,11 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
     </font>
   </fonts>
   <fills count="6">
@@ -187,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -310,6 +315,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -821,7 +829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -913,9 +921,8 @@
           <t>Preço atual</t>
         </is>
       </c>
-      <c r="B7" s="34">
-        <f>'Valuation'!I7</f>
-        <v/>
+      <c r="B7" s="34" t="n">
+        <v>4.26</v>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
@@ -947,9 +954,8 @@
           <t>Preço justo base</t>
         </is>
       </c>
-      <c r="B8" s="34">
-        <f>'Valuation'!H7</f>
-        <v/>
+      <c r="B8" s="34" t="n">
+        <v>4.826334854394739</v>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
@@ -981,9 +987,8 @@
           <t>Upside / Downside</t>
         </is>
       </c>
-      <c r="B9" s="35">
-        <f>'Valuation'!J7</f>
-        <v/>
+      <c r="B9" s="35" t="n">
+        <v>0.1329424540832722</v>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
@@ -1015,9 +1020,8 @@
           <t>EV/EBITDA aplicado</t>
         </is>
       </c>
-      <c r="B10" s="36">
-        <f>'Valuation'!B7</f>
-        <v/>
+      <c r="B10" s="36" t="n">
+        <v>7.398</v>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
@@ -1037,9 +1041,8 @@
           <t>GMAT3 EV/EBITDA atual</t>
         </is>
       </c>
-      <c r="B11" s="36">
-        <f>'Multiplos'!E6</f>
-        <v/>
+      <c r="B11" s="36" t="n">
+        <v>6.583877119999999</v>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
@@ -1059,9 +1062,8 @@
           <t>GMAT3 P/L</t>
         </is>
       </c>
-      <c r="B12" s="36">
-        <f>'Multiplos'!F6</f>
-        <v/>
+      <c r="B12" s="36" t="n">
+        <v>11.50023872300469</v>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
@@ -1074,6 +1076,13 @@
       <c r="G12" s="32" t="n"/>
       <c r="H12" s="32" t="n"/>
       <c r="I12" s="32" t="n"/>
+    </row>
+    <row r="13">
+      <c r="C13" s="45" t="inlineStr">
+        <is>
+          <t>Nota: os valores do resumo são exibidos como outputs finais para evitar cache zerado em visualizadores. A aba Valuation mantém as fórmulas completas da ponte EV → Equity.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>